<commit_message>
vault backup: 2026-09-18 18:27:44
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/02_경영지원_대외비/지출계획_2026-09-18.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/02_경영지원_대외비/지출계획_2026-09-18.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -660,22 +660,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>경영-20260918-005</t>
+          <t>건강-20260918-003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>경영</t>
+          <t>건강</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>경영지원팀</t>
+          <t>건강사업팀</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>김수희</t>
+          <t>전은신</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -693,20 +693,20 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>메트라이프</t>
+          <t>네이버SA&amp;GFA</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>달러경영인정기보험_63회차/55회차</t>
+          <t>네이버 SA&amp;GFA 광고비 충전</t>
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>4900000</v>
+        <v>3498000</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>자동이체</t>
+          <t>계좌송금</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -721,34 +721,29 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>환율에 따라 금액 변경</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>세금·보험(대외비)</t>
+          <t>화/수 2일치 금액</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>경영-20260918-006</t>
+          <t>건강-20260918-004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>경영</t>
+          <t>건강</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>경영지원팀</t>
+          <t>건강사업팀</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>김수희</t>
+          <t>전은신</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -757,7 +752,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -766,20 +761,20 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>SK브로드밴드</t>
+          <t>인포크비즈니스</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>사내전화</t>
+          <t>베리시톨 인플루언서 비용</t>
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>220000</v>
+        <v>3300000</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>자동이체</t>
+          <t>계좌송금</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -792,31 +787,31 @@
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>기타 대외비 지출</t>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>월요일 전부 완성 예상, 재결제 요청 예정</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>건강-20260918-002</t>
+          <t>경영-20260918-005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>건강</t>
+          <t>경영</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>건강사업팀</t>
+          <t>경영지원팀</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>양혜원</t>
+          <t>김수희</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -825,46 +820,56 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>메트라이프</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>네이버 톡톡 발송</t>
+          <t>달러경영인정기보험_63회차/55회차</t>
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>500000</v>
+        <v>4900000</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>계좌송금</t>
+          <t>자동이체</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>신규</t>
+          <t>변경</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
           <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>환율에 따라 금액 변경</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>세금·보험(대외비)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>경영-20260918-007</t>
+          <t>경영-20260918-006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -879,7 +884,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>송채은</t>
+          <t>김수희</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -888,61 +893,66 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>와이투홀딩스</t>
+          <t>SK브로드밴드</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>직원 추석 선물세트 구입</t>
+          <t>사내전화</t>
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>1023110</v>
+        <v>220000</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>계좌송금</t>
+          <t>자동이체</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>변경</t>
+          <t>신규</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
           <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>기타 대외비 지출</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>경영-20260918-003</t>
+          <t>건강-20260918-002</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>경영</t>
+          <t>건강</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>경영지원팀</t>
+          <t>건강사업팀</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>김수희</t>
+          <t>양혜원</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -951,29 +961,29 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>농협카드</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>8월 카드대금</t>
+          <t>네이버 톡톡 발송</t>
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>6827883</v>
+        <v>500000</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>자동이체</t>
+          <t>계좌송금</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -984,18 +994,13 @@
       <c r="N8" t="inlineStr">
         <is>
           <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>기타 대외비 지출</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>경영-20260918-004</t>
+          <t>경영-20260918-007</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1010,7 +1015,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>김수희</t>
+          <t>송채은</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1019,66 +1024,61 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>우리카드</t>
+          <t>와이투홀딩스</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>8월 우리카드 카드대금</t>
+          <t>직원 추석 선물세트 구입</t>
         </is>
       </c>
       <c r="J9" s="2" t="n">
-        <v>25346349</v>
+        <v>1023110</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>자동이체</t>
+          <t>계좌송금</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>신규</t>
+          <t>변경</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
           <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>기타 대외비 지출</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>경영-20260918-012</t>
+          <t>건강-20260918-005</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>경영</t>
+          <t>건강</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>경영지원팀</t>
+          <t>건강사업팀</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>송채은</t>
+          <t>전은신</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1096,16 +1096,16 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>비씨카드</t>
+          <t>써치엠</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>8월카드대금</t>
+          <t>메타 광고 대행 수수</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>269810</v>
+        <v>1487786</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>에이팜</t>
+          <t>8월 광고비에 대한 수수료 11%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>경영-20260918-008</t>
+          <t>건강-20260918-006</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>경영</t>
+          <t>건강</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>경영지원팀</t>
+          <t>건강사업팀</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>김수희</t>
+          <t>전은신</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1155,29 +1155,29 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>메트라이프</t>
+          <t>네이버SA&amp;GFA</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>정기보험_42회차</t>
+          <t>네이버SA&amp;GFA 광고 비용 충전</t>
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>2497000</v>
+        <v>8305000</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>자동이체</t>
+          <t>계좌송금</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1190,31 +1190,31 @@
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>세금·보험(대외비)</t>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>금주 목~차주 월까지 광고비 충전 금액</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>경영-20260918-009</t>
+          <t>건강-20260918-007</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>경영</t>
+          <t>건강</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>경영지원팀</t>
+          <t>건강사업팀</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>김수희</t>
+          <t>전은신</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1223,29 +1223,29 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>ADN</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>통신비</t>
+          <t>ADN 광고-추석 유입</t>
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>109450</v>
+        <v>550000</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>자동이체</t>
+          <t>계좌송금</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1256,18 +1256,13 @@
       <c r="N12" t="inlineStr">
         <is>
           <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>기타 대외비 지출</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>경영-20260918-010</t>
+          <t>경영-20260918-003</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1282,7 +1277,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>송채은</t>
+          <t>김수희</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1291,29 +1286,29 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>서원회계법인</t>
+          <t>농협카드</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>기장료</t>
+          <t>8월 카드대금</t>
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>330000</v>
+        <v>6827883</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>계좌송금</t>
+          <t>자동이체</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1326,16 +1321,16 @@
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>에이팜</t>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>기타 대외비 지출</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>경영-20260918-013</t>
+          <t>경영-20260918-004</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1350,7 +1345,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>송채은</t>
+          <t>김수희</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1359,29 +1354,29 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>가가사무기</t>
+          <t>우리카드</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>복합기 9월 임대비용</t>
+          <t>8월 우리카드 카드대금</t>
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>280000</v>
+        <v>25346349</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>계좌송금</t>
+          <t>자동이체</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1394,75 +1389,415 @@
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>에이팜</t>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>기타 대외비 지출</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>경영-20260918-012</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>경영</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>경영지원팀</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>송채은</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>12</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>비씨카드</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>8월카드대금</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>269810</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>계좌송금</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>에이팜</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>경영-20260918-008</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>경영</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>경영지원팀</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>김수희</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>메트라이프</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>정기보험_42회차</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>2497000</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>자동이체</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>세금·보험(대외비)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>경영-20260918-009</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>경영</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>경영지원팀</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>김수희</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>9</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>통신비</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>109450</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>자동이체</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>기타 대외비 지출</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>경영-20260918-010</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>경영</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>경영지원팀</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>송채은</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>10</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>서원회계법인</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>기장료</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>330000</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>계좌송금</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>에이팜</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>경영-20260918-013</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>경영</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>경영지원팀</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>송채은</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>13</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>가가사무기</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>복합기 9월 임대비용</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>280000</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>계좌송금</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>에이팜</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>경영-20260918-014</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>경영</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>경영지원팀</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>송채은</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
         <v>14</v>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>대구상공회의소</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>하반기연회비</t>
         </is>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="J20" s="2" t="n">
         <v>250000</v>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>계좌송금</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>신규</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
         <is>
           <t>에이팜</t>
         </is>

</xml_diff>

<commit_message>
vault backup: 2026-09-18 21:20:25
</commit_message>
<xml_diff>
--- a/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/02_경영지원_대외비/지출계획_2026-09-18.xlsx
+++ b/01-Projects/에이팜건강-주간자금계획-자동화/자금계획_자동화/02_경영지원_대외비/지출계획_2026-09-18.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1063,22 +1063,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>건강-20260918-005</t>
+          <t>경영-20260918-015</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>건강</t>
+          <t>경영</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>건강사업팀</t>
+          <t>경영지원팀</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>전은신</t>
+          <t>김정원</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1087,25 +1087,25 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>써치엠</t>
+          <t>엠에스바이오텍</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>메타 광고 대행 수수</t>
+          <t>외상매입금</t>
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>1487786</v>
+        <v>20000000</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1124,14 +1124,19 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>8월 광고비에 대한 수수료 11%</t>
+          <t>외상매입금 1차 지급</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>기타 대외비 지출</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>건강-20260918-006</t>
+          <t>건강-20260918-005</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1155,7 +1160,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1164,16 +1169,16 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>네이버SA&amp;GFA</t>
+          <t>써치엠</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>네이버SA&amp;GFA 광고 비용 충전</t>
+          <t>메타 광고 대행 수수</t>
         </is>
       </c>
       <c r="J11" s="2" t="n">
-        <v>8305000</v>
+        <v>1487786</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1192,14 +1197,14 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>금주 목~차주 월까지 광고비 충전 금액</t>
+          <t>8월 광고비에 대한 수수료 11%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>건강-20260918-007</t>
+          <t>건강-20260918-006</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1223,7 +1228,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1232,16 +1237,16 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>ADN</t>
+          <t>네이버SA&amp;GFA</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>ADN 광고-추석 유입</t>
+          <t>네이버SA&amp;GFA 광고 비용 충전</t>
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>550000</v>
+        <v>8305000</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1256,28 +1261,33 @@
       <c r="N12" t="inlineStr">
         <is>
           <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>금주 목~차주 월까지 광고비 충전 금액</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>경영-20260918-003</t>
+          <t>건강-20260918-007</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>경영</t>
+          <t>건강</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>경영지원팀</t>
+          <t>건강사업팀</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>김수희</t>
+          <t>전은신</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1286,7 +1296,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1295,20 +1305,20 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>농협카드</t>
+          <t>ADN</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>8월 카드대금</t>
+          <t>ADN 광고-추석 유입</t>
         </is>
       </c>
       <c r="J13" s="2" t="n">
-        <v>6827883</v>
+        <v>550000</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>자동이체</t>
+          <t>계좌송금</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1319,18 +1329,13 @@
       <c r="N13" t="inlineStr">
         <is>
           <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>기타 대외비 지출</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>경영-20260918-004</t>
+          <t>경영-20260918-003</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1354,7 +1359,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1363,16 +1368,16 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>우리카드</t>
+          <t>농협카드</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>8월 우리카드 카드대금</t>
+          <t>8월 카드대금</t>
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>25346349</v>
+        <v>6827883</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1398,7 +1403,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>경영-20260918-012</t>
+          <t>경영-20260918-004</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1413,7 +1418,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>송채은</t>
+          <t>김수희</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1422,7 +1427,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1431,20 +1436,20 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>비씨카드</t>
+          <t>우리카드</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>8월카드대금</t>
+          <t>8월 우리카드 카드대금</t>
         </is>
       </c>
       <c r="J15" s="2" t="n">
-        <v>269810</v>
+        <v>25346349</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>계좌송금</t>
+          <t>자동이체</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1457,16 +1462,16 @@
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>에이팜</t>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>기타 대외비 지출</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>경영-20260918-008</t>
+          <t>경영-20260918-012</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1481,7 +1486,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>김수희</t>
+          <t>송채은</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1490,29 +1495,29 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>메트라이프</t>
+          <t>비씨카드</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>정기보험_42회차</t>
+          <t>8월카드대금</t>
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>2497000</v>
+        <v>269810</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>자동이체</t>
+          <t>계좌송금</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1525,16 +1530,16 @@
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>세금·보험(대외비)</t>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>에이팜</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>경영-20260918-009</t>
+          <t>경영-20260918-008</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1558,7 +1563,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1567,16 +1572,16 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>KT</t>
+          <t>메트라이프</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>통신비</t>
+          <t>정기보험_42회차</t>
         </is>
       </c>
       <c r="J17" s="2" t="n">
-        <v>109450</v>
+        <v>2497000</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1595,14 +1600,14 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>기타 대외비 지출</t>
+          <t>세금·보험(대외비)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>경영-20260918-010</t>
+          <t>경영-20260918-009</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1617,7 +1622,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>송채은</t>
+          <t>김수희</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1626,29 +1631,29 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>서원회계법인</t>
+          <t>KT</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>기장료</t>
+          <t>통신비</t>
         </is>
       </c>
       <c r="J18" s="2" t="n">
-        <v>330000</v>
+        <v>109450</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>계좌송금</t>
+          <t>자동이체</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1661,16 +1666,16 @@
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>에이팜</t>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>기타 대외비 지출</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>경영-20260918-013</t>
+          <t>경영-20260918-010</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1694,7 +1699,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1703,16 +1708,16 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>가가사무기</t>
+          <t>서원회계법인</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>복합기 9월 임대비용</t>
+          <t>기장료</t>
         </is>
       </c>
       <c r="J19" s="2" t="n">
-        <v>280000</v>
+        <v>330000</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -1738,66 +1743,134 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>경영-20260918-013</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>경영</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>경영지원팀</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>송채은</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>13</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>가가사무기</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>복합기 9월 임대비용</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>280000</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>계좌송금</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>신규</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>에이팜</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>경영-20260918-014</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>경영</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>경영지원팀</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>송채은</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
         <v>14</v>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>대구상공회의소</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>하반기연회비</t>
         </is>
       </c>
-      <c r="J20" s="2" t="n">
+      <c r="J21" s="2" t="n">
         <v>250000</v>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>계좌송금</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>신규</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
         <is>
           <t>에이팜</t>
         </is>

</xml_diff>